<commit_message>
Audit items 1-6: no-ER funds in net series, H3 calibration universe, gap guard, classification base fix, PT common dates; text and tables updated
</commit_message>
<xml_diff>
--- a/data/R import/unknown_classification.xlsx
+++ b/data/R import/unknown_classification.xlsx
@@ -671,17 +671,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2011-12</t>
+          <t>2012-01</t>
         </is>
       </c>
       <c r="G4">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H4">
-        <v>0.294</v>
+        <v>0.042</v>
       </c>
       <c r="I4">
-        <v>14.02</v>
+        <v>48.08</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1188,6 +1188,15 @@
           <t>2001-10</t>
         </is>
       </c>
+      <c r="G12">
+        <v>70</v>
+      </c>
+      <c r="H12">
+        <v>0.803</v>
+      </c>
+      <c r="I12">
+        <v>7.07</v>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
           <t>Active</t>
@@ -1244,6 +1253,9 @@
           <t>2002-01</t>
         </is>
       </c>
+      <c r="G13">
+        <v>9</v>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>Active</t>
@@ -1689,6 +1701,9 @@
           <t>2001-10</t>
         </is>
       </c>
+      <c r="G20">
+        <v>11</v>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
           <t>Active</t>
@@ -2129,6 +2144,9 @@
           <t>2006-09</t>
         </is>
       </c>
+      <c r="G27">
+        <v>6</v>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
           <t>Active</t>
@@ -2499,6 +2517,9 @@
           <t>2009-09</t>
         </is>
       </c>
+      <c r="G33">
+        <v>11</v>
+      </c>
       <c r="J33" t="inlineStr">
         <is>
           <t>Active</t>
@@ -2690,6 +2711,9 @@
           <t>2001-03</t>
         </is>
       </c>
+      <c r="G36">
+        <v>3</v>
+      </c>
       <c r="J36" t="inlineStr">
         <is>
           <t>Active</t>
@@ -3131,6 +3155,15 @@
           <t>2005-06</t>
         </is>
       </c>
+      <c r="G43">
+        <v>30</v>
+      </c>
+      <c r="H43">
+        <v>0.124</v>
+      </c>
+      <c r="I43">
+        <v>12.54</v>
+      </c>
       <c r="J43" t="inlineStr">
         <is>
           <t>Active</t>
@@ -3381,6 +3414,15 @@
           <t>2000-10</t>
         </is>
       </c>
+      <c r="G47">
+        <v>64</v>
+      </c>
+      <c r="H47">
+        <v>0.88</v>
+      </c>
+      <c r="I47">
+        <v>5.25</v>
+      </c>
       <c r="J47" t="inlineStr">
         <is>
           <t>Active</t>
@@ -3567,6 +3609,9 @@
           <t>2009-11</t>
         </is>
       </c>
+      <c r="G50">
+        <v>6</v>
+      </c>
       <c r="J50" t="inlineStr">
         <is>
           <t>Active</t>
@@ -4196,6 +4241,15 @@
           <t>2002-01</t>
         </is>
       </c>
+      <c r="G60">
+        <v>52</v>
+      </c>
+      <c r="H60">
+        <v>0.503</v>
+      </c>
+      <c r="I60">
+        <v>13.48</v>
+      </c>
       <c r="J60" t="inlineStr">
         <is>
           <t>Active</t>
@@ -5667,6 +5721,9 @@
           <t>2001-09</t>
         </is>
       </c>
+      <c r="G83">
+        <v>5</v>
+      </c>
       <c r="J83" t="inlineStr">
         <is>
           <t>Active</t>
@@ -5922,6 +5979,9 @@
           <t>2007-11</t>
         </is>
       </c>
+      <c r="G87">
+        <v>10</v>
+      </c>
       <c r="J87" t="inlineStr">
         <is>
           <t>Active</t>
@@ -6489,17 +6549,17 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2008-09</t>
+          <t>2008-10</t>
         </is>
       </c>
       <c r="G96">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H96">
-        <v>0.447</v>
+        <v>0.002</v>
       </c>
       <c r="I96">
-        <v>10.33</v>
+        <v>21.85</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -7263,17 +7323,17 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2017-04</t>
+          <t>2017-05</t>
         </is>
       </c>
       <c r="G108">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H108">
-        <v>0.012</v>
+        <v>0</v>
       </c>
       <c r="I108">
-        <v>14.06</v>
+        <v>20.92</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
@@ -8167,17 +8227,17 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2018-11</t>
+          <t>2018-12</t>
         </is>
       </c>
       <c r="G122">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H122">
-        <v>0.453</v>
+        <v>0.17</v>
       </c>
       <c r="I122">
-        <v>17.37</v>
+        <v>27.34</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -8742,6 +8802,9 @@
           <t>2016-07</t>
         </is>
       </c>
+      <c r="G131">
+        <v>11</v>
+      </c>
       <c r="J131" t="inlineStr">
         <is>
           <t>Active</t>
@@ -9055,8 +9118,11 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2001-08</t>
-        </is>
+          <t>2001-09</t>
+        </is>
+      </c>
+      <c r="G136">
+        <v>15</v>
       </c>
       <c r="J136" t="inlineStr">
         <is>
@@ -9769,6 +9835,9 @@
           <t>2008-09</t>
         </is>
       </c>
+      <c r="G147">
+        <v>8</v>
+      </c>
       <c r="J147" t="inlineStr">
         <is>
           <t>Active</t>
@@ -9946,17 +10015,17 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="G150">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H150">
-        <v>0.248</v>
+        <v>0.171</v>
       </c>
       <c r="I150">
-        <v>15.78</v>
+        <v>17.82</v>
       </c>
       <c r="J150" t="inlineStr">
         <is>
@@ -10203,6 +10272,9 @@
           <t>2001-08</t>
         </is>
       </c>
+      <c r="G154">
+        <v>11</v>
+      </c>
       <c r="J154" t="inlineStr">
         <is>
           <t>Active</t>
@@ -10766,6 +10838,9 @@
           <t>2001-11</t>
         </is>
       </c>
+      <c r="G163">
+        <v>12</v>
+      </c>
       <c r="J163" t="inlineStr">
         <is>
           <t>Passive</t>
@@ -10893,13 +10968,13 @@
         </is>
       </c>
       <c r="G165">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="H165">
-        <v>0.054</v>
+        <v>0.028</v>
       </c>
       <c r="I165">
-        <v>80.65000000000001</v>
+        <v>98.16</v>
       </c>
       <c r="J165" t="inlineStr">
         <is>
@@ -11087,6 +11162,9 @@
           <t>2007-08</t>
         </is>
       </c>
+      <c r="G168">
+        <v>19</v>
+      </c>
       <c r="J168" t="inlineStr">
         <is>
           <t>Active</t>
@@ -11144,13 +11222,13 @@
         </is>
       </c>
       <c r="G169">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H169">
-        <v>0.859</v>
+        <v>0.407</v>
       </c>
       <c r="I169">
-        <v>10.86</v>
+        <v>34.45</v>
       </c>
       <c r="J169" t="inlineStr">
         <is>
@@ -11205,17 +11283,17 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>2009-04</t>
+          <t>2009-05</t>
         </is>
       </c>
       <c r="G170">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H170">
-        <v>0.4</v>
+        <v>0.27</v>
       </c>
       <c r="I170">
-        <v>14.27</v>
+        <v>17.58</v>
       </c>
       <c r="J170" t="inlineStr">
         <is>
@@ -11533,6 +11611,15 @@
           <t>1999-10</t>
         </is>
       </c>
+      <c r="G175">
+        <v>58</v>
+      </c>
+      <c r="H175">
+        <v>0.821</v>
+      </c>
+      <c r="I175">
+        <v>9.27</v>
+      </c>
       <c r="J175" t="inlineStr">
         <is>
           <t>Active</t>
@@ -11649,6 +11736,9 @@
           <t>2001-03</t>
         </is>
       </c>
+      <c r="G177">
+        <v>4</v>
+      </c>
       <c r="J177" t="inlineStr">
         <is>
           <t>Active</t>
@@ -15513,6 +15603,15 @@
           <t>2006-11</t>
         </is>
       </c>
+      <c r="G237">
+        <v>83</v>
+      </c>
+      <c r="H237">
+        <v>0.408</v>
+      </c>
+      <c r="I237">
+        <v>19.19</v>
+      </c>
       <c r="J237" t="inlineStr">
         <is>
           <t>Active</t>
@@ -15769,6 +15868,15 @@
           <t>2006-11</t>
         </is>
       </c>
+      <c r="G241">
+        <v>83</v>
+      </c>
+      <c r="H241">
+        <v>0.29</v>
+      </c>
+      <c r="I241">
+        <v>18.71</v>
+      </c>
       <c r="J241" t="inlineStr">
         <is>
           <t>Active</t>
@@ -16085,6 +16193,15 @@
           <t>2008-06</t>
         </is>
       </c>
+      <c r="G246">
+        <v>162</v>
+      </c>
+      <c r="H246">
+        <v>0.135</v>
+      </c>
+      <c r="I246">
+        <v>49.95</v>
+      </c>
       <c r="J246" t="inlineStr">
         <is>
           <t>Active</t>
@@ -16340,6 +16457,15 @@
           <t>2001-03</t>
         </is>
       </c>
+      <c r="G250">
+        <v>75</v>
+      </c>
+      <c r="H250">
+        <v>0.542</v>
+      </c>
+      <c r="I250">
+        <v>21.39</v>
+      </c>
       <c r="J250" t="inlineStr">
         <is>
           <t>Active</t>
@@ -16526,6 +16652,9 @@
           <t>2007-03</t>
         </is>
       </c>
+      <c r="G253">
+        <v>14</v>
+      </c>
       <c r="J253" t="inlineStr">
         <is>
           <t>Active</t>
@@ -16787,6 +16916,9 @@
           <t>2012-12</t>
         </is>
       </c>
+      <c r="G257">
+        <v>17</v>
+      </c>
       <c r="J257" t="inlineStr">
         <is>
           <t>Active</t>
@@ -17215,6 +17347,15 @@
           <t>2001-07</t>
         </is>
       </c>
+      <c r="G264">
+        <v>36</v>
+      </c>
+      <c r="H264">
+        <v>0.819</v>
+      </c>
+      <c r="I264">
+        <v>7.53</v>
+      </c>
       <c r="J264" t="inlineStr">
         <is>
           <t>Active</t>
@@ -17541,6 +17682,9 @@
           <t>2012-02</t>
         </is>
       </c>
+      <c r="G269">
+        <v>11</v>
+      </c>
       <c r="J269" t="inlineStr">
         <is>
           <t>Active</t>
@@ -18111,6 +18255,15 @@
           <t>2010-10</t>
         </is>
       </c>
+      <c r="G278">
+        <v>24</v>
+      </c>
+      <c r="H278">
+        <v>0.913</v>
+      </c>
+      <c r="I278">
+        <v>6.74</v>
+      </c>
       <c r="J278" t="inlineStr">
         <is>
           <t>Active</t>
@@ -19255,6 +19408,9 @@
           <t>2016-09</t>
         </is>
       </c>
+      <c r="G296">
+        <v>9</v>
+      </c>
       <c r="J296" t="inlineStr">
         <is>
           <t>Active</t>
@@ -19500,6 +19656,9 @@
           <t>2008-06</t>
         </is>
       </c>
+      <c r="G300">
+        <v>3</v>
+      </c>
       <c r="J300" t="inlineStr">
         <is>
           <t>Active</t>
@@ -19621,6 +19780,15 @@
           <t>2012-10</t>
         </is>
       </c>
+      <c r="G302">
+        <v>214</v>
+      </c>
+      <c r="H302">
+        <v>0.416</v>
+      </c>
+      <c r="I302">
+        <v>29.65</v>
+      </c>
       <c r="J302" t="inlineStr">
         <is>
           <t>Active</t>
@@ -20732,6 +20900,9 @@
           <t>2001-06</t>
         </is>
       </c>
+      <c r="G319">
+        <v>4</v>
+      </c>
       <c r="J319" t="inlineStr">
         <is>
           <t>Passive</t>
@@ -20863,6 +21034,9 @@
           <t>2003-11</t>
         </is>
       </c>
+      <c r="G321">
+        <v>2</v>
+      </c>
       <c r="J321" t="inlineStr">
         <is>
           <t>Active</t>
@@ -21308,6 +21482,15 @@
           <t>2010-05</t>
         </is>
       </c>
+      <c r="G328">
+        <v>102</v>
+      </c>
+      <c r="H328">
+        <v>0.319</v>
+      </c>
+      <c r="I328">
+        <v>13.76</v>
+      </c>
       <c r="J328" t="inlineStr">
         <is>
           <t>Active</t>
@@ -22770,6 +22953,9 @@
           <t>2012-10</t>
         </is>
       </c>
+      <c r="G351">
+        <v>12</v>
+      </c>
       <c r="J351" t="inlineStr">
         <is>
           <t>Active</t>
@@ -23792,6 +23978,9 @@
           <t>2008-05</t>
         </is>
       </c>
+      <c r="G367">
+        <v>7</v>
+      </c>
       <c r="J367" t="inlineStr">
         <is>
           <t>Active</t>
@@ -24214,6 +24403,15 @@
           <t>2001-04</t>
         </is>
       </c>
+      <c r="G374">
+        <v>32</v>
+      </c>
+      <c r="H374">
+        <v>0.638</v>
+      </c>
+      <c r="I374">
+        <v>11.33</v>
+      </c>
       <c r="J374" t="inlineStr">
         <is>
           <t>Active</t>
@@ -24995,6 +25193,9 @@
           <t>2012-12</t>
         </is>
       </c>
+      <c r="G386">
+        <v>20</v>
+      </c>
       <c r="J386" t="inlineStr">
         <is>
           <t>Active</t>
@@ -25895,6 +26096,15 @@
           <t>2009-01</t>
         </is>
       </c>
+      <c r="G400">
+        <v>29</v>
+      </c>
+      <c r="H400">
+        <v>0.854</v>
+      </c>
+      <c r="I400">
+        <v>7.4</v>
+      </c>
       <c r="J400" t="inlineStr">
         <is>
           <t>Active</t>
@@ -26080,6 +26290,15 @@
           <t>2010-12</t>
         </is>
       </c>
+      <c r="G403">
+        <v>59</v>
+      </c>
+      <c r="H403">
+        <v>0.948</v>
+      </c>
+      <c r="I403">
+        <v>4.92</v>
+      </c>
       <c r="J403" t="inlineStr">
         <is>
           <t>Active</t>
@@ -26574,6 +26793,15 @@
           <t>2010-02</t>
         </is>
       </c>
+      <c r="G411">
+        <v>153</v>
+      </c>
+      <c r="H411">
+        <v>0.333</v>
+      </c>
+      <c r="I411">
+        <v>38.67</v>
+      </c>
       <c r="J411" t="inlineStr">
         <is>
           <t>Active</t>
@@ -26700,6 +26928,15 @@
           <t>2002-03</t>
         </is>
       </c>
+      <c r="G413">
+        <v>27</v>
+      </c>
+      <c r="H413">
+        <v>0.95</v>
+      </c>
+      <c r="I413">
+        <v>4.02</v>
+      </c>
       <c r="J413" t="inlineStr">
         <is>
           <t>Active</t>
@@ -27151,6 +27388,9 @@
           <t>2012-11</t>
         </is>
       </c>
+      <c r="G420">
+        <v>11</v>
+      </c>
       <c r="J420" t="inlineStr">
         <is>
           <t>Active</t>
@@ -27471,6 +27711,9 @@
           <t>2003-02</t>
         </is>
       </c>
+      <c r="G425">
+        <v>7</v>
+      </c>
       <c r="J425" t="inlineStr">
         <is>
           <t>Active</t>
@@ -27584,17 +27827,17 @@
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t>2008-10</t>
+          <t>2008-11</t>
         </is>
       </c>
       <c r="G427">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H427">
-        <v>0.593</v>
+        <v>0.537</v>
       </c>
       <c r="I427">
-        <v>11.48</v>
+        <v>14.17</v>
       </c>
       <c r="J427" t="inlineStr">
         <is>
@@ -27783,17 +28026,17 @@
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>2001-09</t>
+          <t>2001-10</t>
         </is>
       </c>
       <c r="G430">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H430">
-        <v>0.6919999999999999</v>
+        <v>0.334</v>
       </c>
       <c r="I430">
-        <v>11.89</v>
+        <v>19.17</v>
       </c>
       <c r="J430" t="inlineStr">
         <is>
@@ -28441,6 +28684,9 @@
           <t>2011-11</t>
         </is>
       </c>
+      <c r="G440">
+        <v>4</v>
+      </c>
       <c r="J440" t="inlineStr">
         <is>
           <t>Active</t>
@@ -28626,6 +28872,15 @@
           <t>2011-12</t>
         </is>
       </c>
+      <c r="G443">
+        <v>73</v>
+      </c>
+      <c r="H443">
+        <v>0.533</v>
+      </c>
+      <c r="I443">
+        <v>13.03</v>
+      </c>
       <c r="J443" t="inlineStr">
         <is>
           <t>Active</t>
@@ -29861,6 +30116,9 @@
           <t>2002-09</t>
         </is>
       </c>
+      <c r="G462">
+        <v>17</v>
+      </c>
       <c r="J462" t="inlineStr">
         <is>
           <t>Active</t>
@@ -30809,6 +31067,15 @@
           <t>2001-06</t>
         </is>
       </c>
+      <c r="G477">
+        <v>47</v>
+      </c>
+      <c r="H477">
+        <v>0.295</v>
+      </c>
+      <c r="I477">
+        <v>16.41</v>
+      </c>
       <c r="J477" t="inlineStr">
         <is>
           <t>Active</t>
@@ -30870,6 +31137,9 @@
           <t>2002-02</t>
         </is>
       </c>
+      <c r="G478">
+        <v>19</v>
+      </c>
       <c r="J478" t="inlineStr">
         <is>
           <t>Active</t>
@@ -31837,17 +32107,17 @@
       </c>
       <c r="F493" t="inlineStr">
         <is>
-          <t>2007-02</t>
+          <t>2007-03</t>
         </is>
       </c>
       <c r="G493">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H493">
-        <v>0.6820000000000001</v>
+        <v>0.139</v>
       </c>
       <c r="I493">
-        <v>15.1</v>
+        <v>33.56</v>
       </c>
       <c r="J493" t="inlineStr">
         <is>
@@ -31905,6 +32175,9 @@
           <t>2019-02</t>
         </is>
       </c>
+      <c r="G494">
+        <v>12</v>
+      </c>
       <c r="J494" t="inlineStr">
         <is>
           <t>Active</t>
@@ -31961,6 +32234,15 @@
           <t>2011-03</t>
         </is>
       </c>
+      <c r="G495">
+        <v>38</v>
+      </c>
+      <c r="H495">
+        <v>0.99</v>
+      </c>
+      <c r="I495">
+        <v>2.34</v>
+      </c>
       <c r="J495" t="inlineStr">
         <is>
           <t>Active</t>
@@ -32401,6 +32683,9 @@
           <t>2016-06</t>
         </is>
       </c>
+      <c r="G502">
+        <v>8</v>
+      </c>
       <c r="J502" t="inlineStr">
         <is>
           <t>Active</t>
@@ -32657,6 +32942,9 @@
           <t>2003-07</t>
         </is>
       </c>
+      <c r="G506">
+        <v>11</v>
+      </c>
       <c r="J506" t="inlineStr">
         <is>
           <t>Active</t>
@@ -34007,6 +34295,15 @@
           <t>2006-11</t>
         </is>
       </c>
+      <c r="G527">
+        <v>118</v>
+      </c>
+      <c r="H527">
+        <v>0.323</v>
+      </c>
+      <c r="I527">
+        <v>20.6</v>
+      </c>
       <c r="J527" t="inlineStr">
         <is>
           <t>Active</t>
@@ -35432,6 +35729,15 @@
           <t>2009-04</t>
         </is>
       </c>
+      <c r="G549">
+        <v>29</v>
+      </c>
+      <c r="H549">
+        <v>0.711</v>
+      </c>
+      <c r="I549">
+        <v>23.1</v>
+      </c>
       <c r="J549" t="inlineStr">
         <is>
           <t>Active</t>
@@ -35488,6 +35794,9 @@
           <t>2009-05</t>
         </is>
       </c>
+      <c r="G550">
+        <v>13</v>
+      </c>
       <c r="J550" t="inlineStr">
         <is>
           <t>Active</t>
@@ -35744,6 +36053,15 @@
           <t>2005-06</t>
         </is>
       </c>
+      <c r="G554">
+        <v>54</v>
+      </c>
+      <c r="H554">
+        <v>0.524</v>
+      </c>
+      <c r="I554">
+        <v>19.16</v>
+      </c>
       <c r="J554" t="inlineStr">
         <is>
           <t>Active</t>
@@ -37123,6 +37441,9 @@
           <t>2009-02</t>
         </is>
       </c>
+      <c r="G575">
+        <v>11</v>
+      </c>
       <c r="J575" t="inlineStr">
         <is>
           <t>Active</t>
@@ -37438,6 +37759,9 @@
           <t>2001-10</t>
         </is>
       </c>
+      <c r="G580">
+        <v>10</v>
+      </c>
       <c r="J580" t="inlineStr">
         <is>
           <t>Active</t>
@@ -37491,11 +37815,17 @@
       </c>
       <c r="F581" t="inlineStr">
         <is>
-          <t>2013-06</t>
+          <t>2013-07</t>
         </is>
       </c>
       <c r="G581">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="H581">
+        <v>0.223</v>
+      </c>
+      <c r="I581">
+        <v>26.02</v>
       </c>
       <c r="J581" t="inlineStr">
         <is>
@@ -38072,6 +38402,15 @@
           <t>2002-02</t>
         </is>
       </c>
+      <c r="G590">
+        <v>47</v>
+      </c>
+      <c r="H590">
+        <v>0.667</v>
+      </c>
+      <c r="I590">
+        <v>15.17</v>
+      </c>
       <c r="J590" t="inlineStr">
         <is>
           <t>Active</t>
@@ -38523,6 +38862,9 @@
           <t>2009-12</t>
         </is>
       </c>
+      <c r="G597">
+        <v>17</v>
+      </c>
       <c r="J597" t="inlineStr">
         <is>
           <t>Active</t>
@@ -38709,6 +39051,9 @@
           <t>2013-11</t>
         </is>
       </c>
+      <c r="G600">
+        <v>8</v>
+      </c>
       <c r="J600" t="inlineStr">
         <is>
           <t>Active</t>
@@ -38944,6 +39289,9 @@
           <t>2001-01</t>
         </is>
       </c>
+      <c r="G604">
+        <v>4</v>
+      </c>
       <c r="J604" t="inlineStr">
         <is>
           <t>Active</t>
@@ -39065,6 +39413,9 @@
           <t>2004-12</t>
         </is>
       </c>
+      <c r="G606">
+        <v>10</v>
+      </c>
       <c r="J606" t="inlineStr">
         <is>
           <t>Active</t>
@@ -40349,6 +40700,9 @@
           <t>2001-06</t>
         </is>
       </c>
+      <c r="G626">
+        <v>3</v>
+      </c>
       <c r="J626" t="inlineStr">
         <is>
           <t>Active</t>
@@ -40475,6 +40829,9 @@
           <t>2004-05</t>
         </is>
       </c>
+      <c r="G628">
+        <v>16</v>
+      </c>
       <c r="J628" t="inlineStr">
         <is>
           <t>Active</t>
@@ -41164,13 +41521,13 @@
         </is>
       </c>
       <c r="G639">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H639">
-        <v>0.639</v>
+        <v>0.022</v>
       </c>
       <c r="I639">
-        <v>12.51</v>
+        <v>62.78</v>
       </c>
       <c r="J639" t="inlineStr">
         <is>
@@ -42247,6 +42604,15 @@
           <t>2006-12</t>
         </is>
       </c>
+      <c r="G656">
+        <v>118</v>
+      </c>
+      <c r="H656">
+        <v>0.724</v>
+      </c>
+      <c r="I656">
+        <v>19.7</v>
+      </c>
       <c r="J656" t="inlineStr">
         <is>
           <t>Active</t>
@@ -42438,6 +42804,15 @@
           <t>2001-02</t>
         </is>
       </c>
+      <c r="G659">
+        <v>42</v>
+      </c>
+      <c r="H659">
+        <v>0.946</v>
+      </c>
+      <c r="I659">
+        <v>4.22</v>
+      </c>
       <c r="J659" t="inlineStr">
         <is>
           <t>Active</t>
@@ -42559,6 +42934,9 @@
           <t>2001-11</t>
         </is>
       </c>
+      <c r="G661">
+        <v>7</v>
+      </c>
       <c r="J661" t="inlineStr">
         <is>
           <t>Active</t>
@@ -44906,6 +45284,15 @@
           <t>2011-03</t>
         </is>
       </c>
+      <c r="G697">
+        <v>38</v>
+      </c>
+      <c r="H697">
+        <v>0.9360000000000001</v>
+      </c>
+      <c r="I697">
+        <v>5.87</v>
+      </c>
       <c r="J697" t="inlineStr">
         <is>
           <t>Active</t>
@@ -44962,6 +45349,15 @@
           <t>2011-04</t>
         </is>
       </c>
+      <c r="G698">
+        <v>40</v>
+      </c>
+      <c r="H698">
+        <v>0.851</v>
+      </c>
+      <c r="I698">
+        <v>11.6</v>
+      </c>
       <c r="J698" t="inlineStr">
         <is>
           <t>Active</t>
@@ -45278,6 +45674,9 @@
           <t>2009-04</t>
         </is>
       </c>
+      <c r="G703">
+        <v>17</v>
+      </c>
       <c r="J703" t="inlineStr">
         <is>
           <t>Active</t>
@@ -46048,13 +46447,13 @@
         </is>
       </c>
       <c r="G715">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H715">
-        <v>0.417</v>
+        <v>0.246</v>
       </c>
       <c r="I715">
-        <v>20.86</v>
+        <v>27.27</v>
       </c>
       <c r="J715" t="inlineStr">
         <is>
@@ -46437,6 +46836,9 @@
           <t>2012-07</t>
         </is>
       </c>
+      <c r="G721">
+        <v>23</v>
+      </c>
       <c r="J721" t="inlineStr">
         <is>
           <t>Active</t>
@@ -46623,6 +47025,9 @@
           <t>2012-08</t>
         </is>
       </c>
+      <c r="G724">
+        <v>11</v>
+      </c>
       <c r="J724" t="inlineStr">
         <is>
           <t>Active</t>
@@ -47723,6 +48128,9 @@
           <t>2010-12</t>
         </is>
       </c>
+      <c r="G741">
+        <v>9</v>
+      </c>
       <c r="J741" t="inlineStr">
         <is>
           <t>Active</t>
@@ -49145,6 +49553,15 @@
           <t>2011-10</t>
         </is>
       </c>
+      <c r="G763">
+        <v>59</v>
+      </c>
+      <c r="H763">
+        <v>0.93</v>
+      </c>
+      <c r="I763">
+        <v>5.14</v>
+      </c>
       <c r="J763" t="inlineStr">
         <is>
           <t>Active</t>
@@ -49789,6 +50206,9 @@
           <t>2002-06</t>
         </is>
       </c>
+      <c r="G773">
+        <v>3</v>
+      </c>
       <c r="J773" t="inlineStr">
         <is>
           <t>Active</t>
@@ -50040,6 +50460,15 @@
           <t>2009-08</t>
         </is>
       </c>
+      <c r="G777">
+        <v>44</v>
+      </c>
+      <c r="H777">
+        <v>0</v>
+      </c>
+      <c r="I777">
+        <v>20.33</v>
+      </c>
       <c r="J777" t="inlineStr">
         <is>
           <t>Active</t>
@@ -50226,6 +50655,9 @@
           <t>2011-10</t>
         </is>
       </c>
+      <c r="G780">
+        <v>13</v>
+      </c>
       <c r="J780" t="inlineStr">
         <is>
           <t>Active</t>
@@ -51630,6 +52062,15 @@
           <t>2001-09</t>
         </is>
       </c>
+      <c r="G802">
+        <v>81</v>
+      </c>
+      <c r="H802">
+        <v>0.38</v>
+      </c>
+      <c r="I802">
+        <v>14.63</v>
+      </c>
       <c r="J802" t="inlineStr">
         <is>
           <t>Active</t>
@@ -51880,6 +52321,9 @@
           <t>2006-12</t>
         </is>
       </c>
+      <c r="G806">
+        <v>5</v>
+      </c>
       <c r="J806" t="inlineStr">
         <is>
           <t>Active</t>
@@ -52320,6 +52764,15 @@
           <t>2010-10</t>
         </is>
       </c>
+      <c r="G813">
+        <v>33</v>
+      </c>
+      <c r="H813">
+        <v>0.908</v>
+      </c>
+      <c r="I813">
+        <v>9.9</v>
+      </c>
       <c r="J813" t="inlineStr">
         <is>
           <t>Active</t>
@@ -52376,6 +52829,15 @@
           <t>2011-03</t>
         </is>
       </c>
+      <c r="G814">
+        <v>38</v>
+      </c>
+      <c r="H814">
+        <v>0.906</v>
+      </c>
+      <c r="I814">
+        <v>8.08</v>
+      </c>
       <c r="J814" t="inlineStr">
         <is>
           <t>Active</t>
@@ -54118,6 +54580,9 @@
           <t>2012-09</t>
         </is>
       </c>
+      <c r="G841">
+        <v>9</v>
+      </c>
       <c r="J841" t="inlineStr">
         <is>
           <t>Active</t>
@@ -54174,6 +54639,9 @@
           <t>2012-10</t>
         </is>
       </c>
+      <c r="G842">
+        <v>10</v>
+      </c>
       <c r="J842" t="inlineStr">
         <is>
           <t>Active</t>
@@ -54230,6 +54698,9 @@
           <t>2012-10</t>
         </is>
       </c>
+      <c r="G843">
+        <v>10</v>
+      </c>
       <c r="J843" t="inlineStr">
         <is>
           <t>Active</t>
@@ -55258,6 +55729,9 @@
           <t>1999-06</t>
         </is>
       </c>
+      <c r="G859">
+        <v>14</v>
+      </c>
       <c r="J859" t="inlineStr">
         <is>
           <t>Active</t>
@@ -55768,6 +56242,9 @@
           <t>2011-04</t>
         </is>
       </c>
+      <c r="G867">
+        <v>16</v>
+      </c>
       <c r="J867" t="inlineStr">
         <is>
           <t>Active</t>
@@ -57253,6 +57730,15 @@
           <t>2001-11</t>
         </is>
       </c>
+      <c r="G890">
+        <v>66</v>
+      </c>
+      <c r="H890">
+        <v>0.677</v>
+      </c>
+      <c r="I890">
+        <v>12.56</v>
+      </c>
       <c r="J890" t="inlineStr">
         <is>
           <t>Active</t>
@@ -58129,6 +58615,9 @@
           <t>2016-09</t>
         </is>
       </c>
+      <c r="G903">
+        <v>16</v>
+      </c>
       <c r="J903" t="inlineStr">
         <is>
           <t>Active</t>
@@ -58580,6 +59069,15 @@
           <t>2009-03</t>
         </is>
       </c>
+      <c r="G910">
+        <v>30</v>
+      </c>
+      <c r="H910">
+        <v>0.921</v>
+      </c>
+      <c r="I910">
+        <v>6.31</v>
+      </c>
       <c r="J910" t="inlineStr">
         <is>
           <t>Active</t>
@@ -58636,6 +59134,15 @@
           <t>2011-06</t>
         </is>
       </c>
+      <c r="G911">
+        <v>56</v>
+      </c>
+      <c r="H911">
+        <v>0.91</v>
+      </c>
+      <c r="I911">
+        <v>5.65</v>
+      </c>
       <c r="J911" t="inlineStr">
         <is>
           <t>Active</t>
@@ -58876,6 +59383,9 @@
           <t>2018-07</t>
         </is>
       </c>
+      <c r="G915">
+        <v>3</v>
+      </c>
       <c r="J915" t="inlineStr">
         <is>
           <t>Active</t>
@@ -59367,6 +59877,15 @@
           <t>2000-09</t>
         </is>
       </c>
+      <c r="G923">
+        <v>69</v>
+      </c>
+      <c r="H923">
+        <v>0.167</v>
+      </c>
+      <c r="I923">
+        <v>14.85</v>
+      </c>
       <c r="J923" t="inlineStr">
         <is>
           <t>Active</t>
@@ -59688,6 +60207,9 @@
           <t>2014-10</t>
         </is>
       </c>
+      <c r="G928">
+        <v>9</v>
+      </c>
       <c r="J928" t="inlineStr">
         <is>
           <t>Active</t>
@@ -59868,6 +60390,9 @@
           <t>2011-05</t>
         </is>
       </c>
+      <c r="G931">
+        <v>6</v>
+      </c>
       <c r="J931" t="inlineStr">
         <is>
           <t>Active</t>
@@ -59983,6 +60508,9 @@
           <t>2000-09</t>
         </is>
       </c>
+      <c r="G933">
+        <v>7</v>
+      </c>
       <c r="J933" t="inlineStr">
         <is>
           <t>Active</t>
@@ -60168,6 +60696,9 @@
           <t>2010-01</t>
         </is>
       </c>
+      <c r="G936">
+        <v>9</v>
+      </c>
       <c r="J936" t="inlineStr">
         <is>
           <t>Active</t>
@@ -61089,6 +61620,9 @@
           <t>2011-05</t>
         </is>
       </c>
+      <c r="G950">
+        <v>14</v>
+      </c>
       <c r="J950" t="inlineStr">
         <is>
           <t>Active</t>
@@ -61145,6 +61679,15 @@
           <t>1999-12</t>
         </is>
       </c>
+      <c r="G951">
+        <v>60</v>
+      </c>
+      <c r="H951">
+        <v>0.736</v>
+      </c>
+      <c r="I951">
+        <v>9.19</v>
+      </c>
       <c r="J951" t="inlineStr">
         <is>
           <t>Active</t>
@@ -61331,6 +61874,9 @@
           <t>2009-01</t>
         </is>
       </c>
+      <c r="G954">
+        <v>6</v>
+      </c>
       <c r="J954" t="inlineStr">
         <is>
           <t>Active</t>
@@ -61976,6 +62522,15 @@
           <t>2011-06</t>
         </is>
       </c>
+      <c r="G964">
+        <v>33</v>
+      </c>
+      <c r="H964">
+        <v>0.918</v>
+      </c>
+      <c r="I964">
+        <v>6.25</v>
+      </c>
       <c r="J964" t="inlineStr">
         <is>
           <t>Active</t>
@@ -62032,6 +62587,15 @@
           <t>2011-06</t>
         </is>
       </c>
+      <c r="G965">
+        <v>33</v>
+      </c>
+      <c r="H965">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="I965">
+        <v>7.44</v>
+      </c>
       <c r="J965" t="inlineStr">
         <is>
           <t>Active</t>
@@ -62088,6 +62652,15 @@
           <t>2011-12</t>
         </is>
       </c>
+      <c r="G966">
+        <v>61</v>
+      </c>
+      <c r="H966">
+        <v>0.964</v>
+      </c>
+      <c r="I966">
+        <v>4.65</v>
+      </c>
       <c r="J966" t="inlineStr">
         <is>
           <t>Active</t>
@@ -62144,6 +62717,15 @@
           <t>2011-06</t>
         </is>
       </c>
+      <c r="G967">
+        <v>33</v>
+      </c>
+      <c r="H967">
+        <v>0.883</v>
+      </c>
+      <c r="I967">
+        <v>10.14</v>
+      </c>
       <c r="J967" t="inlineStr">
         <is>
           <t>Active</t>
@@ -62259,6 +62841,15 @@
         <is>
           <t>2004-11</t>
         </is>
+      </c>
+      <c r="G969">
+        <v>100</v>
+      </c>
+      <c r="H969">
+        <v>0.54</v>
+      </c>
+      <c r="I969">
+        <v>37.21</v>
       </c>
       <c r="J969" t="inlineStr">
         <is>
@@ -62389,10 +62980,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>2256</v>
+        <v>2255</v>
       </c>
       <c r="C2">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">

</xml_diff>